<commit_message>
fix: update the unique identifier to email, manual modifications of excel files to eliminate uncertainity
</commit_message>
<xml_diff>
--- a/frontend/public/weekly_contest_1_leaderboard.xlsx
+++ b/frontend/public/weekly_contest_1_leaderboard.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="213">
   <si>
     <t>Name</t>
   </si>
@@ -302,12 +302,6 @@
   </si>
   <si>
     <t>dishanaveen18@gmail.com</t>
-  </si>
-  <si>
-    <t>K S Sujesh</t>
-  </si>
-  <si>
-    <t>kssujesh27@gmail.com</t>
   </si>
   <si>
     <t>ANSH VASHISHT</t>
@@ -1741,13 +1735,13 @@
         <v>98</v>
       </c>
       <c r="C48" s="3">
-        <v>350.0</v>
+        <v>340.0</v>
       </c>
       <c r="D48" s="3">
         <v>500.0</v>
       </c>
       <c r="E48" s="4">
-        <v>0.05974537037037037</v>
+        <v>0.012824074074074075</v>
       </c>
     </row>
     <row r="49">
@@ -1764,7 +1758,7 @@
         <v>500.0</v>
       </c>
       <c r="E49" s="4">
-        <v>0.012824074074074075</v>
+        <v>0.05101851851851852</v>
       </c>
     </row>
     <row r="50">
@@ -1775,13 +1769,13 @@
         <v>102</v>
       </c>
       <c r="C50" s="3">
-        <v>340.0</v>
+        <v>320.0</v>
       </c>
       <c r="D50" s="3">
         <v>500.0</v>
       </c>
       <c r="E50" s="4">
-        <v>0.05101851851851852</v>
+        <v>0.062453703703703706</v>
       </c>
     </row>
     <row r="51">
@@ -1792,13 +1786,13 @@
         <v>104</v>
       </c>
       <c r="C51" s="3">
-        <v>320.0</v>
+        <v>280.0</v>
       </c>
       <c r="D51" s="3">
         <v>500.0</v>
       </c>
       <c r="E51" s="4">
-        <v>0.062453703703703706</v>
+        <v>0.03304398148148148</v>
       </c>
     </row>
     <row r="52">
@@ -1809,13 +1803,13 @@
         <v>106</v>
       </c>
       <c r="C52" s="3">
-        <v>280.0</v>
+        <v>200.0</v>
       </c>
       <c r="D52" s="3">
         <v>500.0</v>
       </c>
       <c r="E52" s="4">
-        <v>0.03304398148148148</v>
+        <v>0.020833333333333332</v>
       </c>
     </row>
     <row r="53">
@@ -1832,7 +1826,7 @@
         <v>500.0</v>
       </c>
       <c r="E53" s="4">
-        <v>0.020833333333333332</v>
+        <v>0.03200231481481482</v>
       </c>
     </row>
     <row r="54">
@@ -1849,7 +1843,7 @@
         <v>500.0</v>
       </c>
       <c r="E54" s="4">
-        <v>0.03200231481481482</v>
+        <v>0.03325231481481482</v>
       </c>
     </row>
     <row r="55">
@@ -1866,7 +1860,7 @@
         <v>500.0</v>
       </c>
       <c r="E55" s="4">
-        <v>0.03325231481481482</v>
+        <v>0.03581018518518519</v>
       </c>
     </row>
     <row r="56">
@@ -1883,7 +1877,7 @@
         <v>500.0</v>
       </c>
       <c r="E56" s="4">
-        <v>0.03581018518518519</v>
+        <v>0.049652777777777775</v>
       </c>
     </row>
     <row r="57">
@@ -1900,7 +1894,7 @@
         <v>500.0</v>
       </c>
       <c r="E57" s="4">
-        <v>0.049652777777777775</v>
+        <v>0.051041666666666666</v>
       </c>
     </row>
     <row r="58">
@@ -1917,7 +1911,7 @@
         <v>500.0</v>
       </c>
       <c r="E58" s="4">
-        <v>0.051041666666666666</v>
+        <v>0.05552083333333333</v>
       </c>
     </row>
     <row r="59">
@@ -1934,7 +1928,7 @@
         <v>500.0</v>
       </c>
       <c r="E59" s="4">
-        <v>0.05552083333333333</v>
+        <v>0.061828703703703705</v>
       </c>
     </row>
     <row r="60">
@@ -1951,7 +1945,7 @@
         <v>500.0</v>
       </c>
       <c r="E60" s="4">
-        <v>0.061828703703703705</v>
+        <v>0.06189814814814815</v>
       </c>
     </row>
     <row r="61">
@@ -1968,7 +1962,7 @@
         <v>500.0</v>
       </c>
       <c r="E61" s="4">
-        <v>0.06189814814814815</v>
+        <v>0.06208333333333333</v>
       </c>
     </row>
     <row r="62">
@@ -1979,13 +1973,13 @@
         <v>126</v>
       </c>
       <c r="C62" s="3">
-        <v>200.0</v>
+        <v>180.0</v>
       </c>
       <c r="D62" s="3">
         <v>500.0</v>
       </c>
       <c r="E62" s="4">
-        <v>0.06208333333333333</v>
+        <v>0.028136574074074074</v>
       </c>
     </row>
     <row r="63">
@@ -2002,7 +1996,7 @@
         <v>500.0</v>
       </c>
       <c r="E63" s="4">
-        <v>0.028136574074074074</v>
+        <v>0.05693287037037037</v>
       </c>
     </row>
     <row r="64">
@@ -2019,7 +2013,7 @@
         <v>500.0</v>
       </c>
       <c r="E64" s="4">
-        <v>0.05693287037037037</v>
+        <v>0.06251157407407408</v>
       </c>
     </row>
     <row r="65">
@@ -2030,13 +2024,13 @@
         <v>132</v>
       </c>
       <c r="C65" s="3">
-        <v>180.0</v>
+        <v>150.0</v>
       </c>
       <c r="D65" s="3">
         <v>500.0</v>
       </c>
       <c r="E65" s="4">
-        <v>0.06251157407407408</v>
+        <v>0.024965277777777777</v>
       </c>
     </row>
     <row r="66">
@@ -2047,13 +2041,13 @@
         <v>134</v>
       </c>
       <c r="C66" s="3">
-        <v>150.0</v>
+        <v>110.0</v>
       </c>
       <c r="D66" s="3">
         <v>500.0</v>
       </c>
       <c r="E66" s="4">
-        <v>0.024965277777777777</v>
+        <v>0.052314814814814814</v>
       </c>
     </row>
     <row r="67">
@@ -2064,13 +2058,13 @@
         <v>136</v>
       </c>
       <c r="C67" s="3">
-        <v>110.0</v>
+        <v>80.0</v>
       </c>
       <c r="D67" s="3">
         <v>500.0</v>
       </c>
       <c r="E67" s="4">
-        <v>0.052314814814814814</v>
+        <v>0.050520833333333334</v>
       </c>
     </row>
     <row r="68">
@@ -2081,13 +2075,13 @@
         <v>138</v>
       </c>
       <c r="C68" s="3">
-        <v>80.0</v>
+        <v>70.0</v>
       </c>
       <c r="D68" s="3">
         <v>500.0</v>
       </c>
       <c r="E68" s="4">
-        <v>0.050520833333333334</v>
+        <v>0.0577662037037037</v>
       </c>
     </row>
     <row r="69">
@@ -2104,7 +2098,7 @@
         <v>500.0</v>
       </c>
       <c r="E69" s="4">
-        <v>0.0577662037037037</v>
+        <v>0.06251157407407408</v>
       </c>
     </row>
     <row r="70">
@@ -2115,13 +2109,13 @@
         <v>142</v>
       </c>
       <c r="C70" s="3">
-        <v>70.0</v>
+        <v>50.0</v>
       </c>
       <c r="D70" s="3">
         <v>500.0</v>
       </c>
       <c r="E70" s="4">
-        <v>0.06251157407407408</v>
+        <v>0.02236111111111111</v>
       </c>
     </row>
     <row r="71">
@@ -2138,7 +2132,7 @@
         <v>500.0</v>
       </c>
       <c r="E71" s="4">
-        <v>0.02236111111111111</v>
+        <v>0.027372685185185184</v>
       </c>
     </row>
     <row r="72">
@@ -2155,15 +2149,15 @@
         <v>500.0</v>
       </c>
       <c r="E72" s="4">
-        <v>0.027372685185185184</v>
+        <v>0.028576388888888887</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B73" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>148</v>
       </c>
       <c r="C73" s="3">
         <v>50.0</v>
@@ -2172,12 +2166,12 @@
         <v>500.0</v>
       </c>
       <c r="E73" s="4">
-        <v>0.028576388888888887</v>
+        <v>0.030694444444444444</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="s">
-        <v>43</v>
+        <v>148</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>149</v>
@@ -2189,7 +2183,7 @@
         <v>500.0</v>
       </c>
       <c r="E74" s="4">
-        <v>0.030694444444444444</v>
+        <v>0.04878472222222222</v>
       </c>
     </row>
     <row r="75">
@@ -2206,7 +2200,7 @@
         <v>500.0</v>
       </c>
       <c r="E75" s="4">
-        <v>0.04878472222222222</v>
+        <v>0.05496527777777778</v>
       </c>
     </row>
     <row r="76">
@@ -2223,7 +2217,7 @@
         <v>500.0</v>
       </c>
       <c r="E76" s="4">
-        <v>0.05496527777777778</v>
+        <v>0.06100694444444445</v>
       </c>
     </row>
     <row r="77">
@@ -2234,13 +2228,13 @@
         <v>155</v>
       </c>
       <c r="C77" s="3">
-        <v>50.0</v>
+        <v>40.0</v>
       </c>
       <c r="D77" s="3">
         <v>500.0</v>
       </c>
       <c r="E77" s="4">
-        <v>0.06100694444444445</v>
+        <v>0.00829861111111111</v>
       </c>
     </row>
     <row r="78">
@@ -2257,7 +2251,7 @@
         <v>500.0</v>
       </c>
       <c r="E78" s="4">
-        <v>0.00829861111111111</v>
+        <v>0.008726851851851852</v>
       </c>
     </row>
     <row r="79">
@@ -2274,7 +2268,7 @@
         <v>500.0</v>
       </c>
       <c r="E79" s="4">
-        <v>0.008726851851851852</v>
+        <v>0.009398148148148149</v>
       </c>
     </row>
     <row r="80">
@@ -2291,7 +2285,7 @@
         <v>500.0</v>
       </c>
       <c r="E80" s="4">
-        <v>0.009398148148148149</v>
+        <v>0.04704861111111111</v>
       </c>
     </row>
     <row r="81">
@@ -2308,7 +2302,7 @@
         <v>500.0</v>
       </c>
       <c r="E81" s="4">
-        <v>0.04704861111111111</v>
+        <v>0.05298611111111111</v>
       </c>
     </row>
     <row r="82">
@@ -2325,7 +2319,7 @@
         <v>500.0</v>
       </c>
       <c r="E82" s="4">
-        <v>0.05298611111111111</v>
+        <v>0.056226851851851854</v>
       </c>
     </row>
     <row r="83">
@@ -2336,13 +2330,13 @@
         <v>167</v>
       </c>
       <c r="C83" s="3">
-        <v>40.0</v>
+        <v>30.0</v>
       </c>
       <c r="D83" s="3">
         <v>500.0</v>
       </c>
       <c r="E83" s="4">
-        <v>0.056226851851851854</v>
+        <v>0.031516203703703706</v>
       </c>
     </row>
     <row r="84">
@@ -2359,7 +2353,7 @@
         <v>500.0</v>
       </c>
       <c r="E84" s="4">
-        <v>0.031516203703703706</v>
+        <v>0.05358796296296296</v>
       </c>
     </row>
     <row r="85">
@@ -2376,7 +2370,7 @@
         <v>500.0</v>
       </c>
       <c r="E85" s="4">
-        <v>0.05358796296296296</v>
+        <v>0.05846064814814815</v>
       </c>
     </row>
     <row r="86">
@@ -2393,7 +2387,7 @@
         <v>500.0</v>
       </c>
       <c r="E86" s="4">
-        <v>0.05846064814814815</v>
+        <v>0.06251157407407408</v>
       </c>
     </row>
     <row r="87">
@@ -2421,13 +2415,13 @@
         <v>177</v>
       </c>
       <c r="C88" s="3">
-        <v>30.0</v>
+        <v>20.0</v>
       </c>
       <c r="D88" s="3">
         <v>500.0</v>
       </c>
       <c r="E88" s="4">
-        <v>0.06251157407407408</v>
+        <v>0.019837962962962963</v>
       </c>
     </row>
     <row r="89">
@@ -2444,7 +2438,7 @@
         <v>500.0</v>
       </c>
       <c r="E89" s="4">
-        <v>0.019837962962962963</v>
+        <v>0.05613425925925926</v>
       </c>
     </row>
     <row r="90">
@@ -2455,13 +2449,13 @@
         <v>181</v>
       </c>
       <c r="C90" s="3">
-        <v>20.0</v>
+        <v>0.0</v>
       </c>
       <c r="D90" s="3">
         <v>500.0</v>
       </c>
       <c r="E90" s="4">
-        <v>0.05613425925925926</v>
+        <v>0.0059722222222222225</v>
       </c>
     </row>
     <row r="91">
@@ -2478,7 +2472,7 @@
         <v>500.0</v>
       </c>
       <c r="E91" s="4">
-        <v>0.0059722222222222225</v>
+        <v>0.006504629629629629</v>
       </c>
     </row>
     <row r="92">
@@ -2495,7 +2489,7 @@
         <v>500.0</v>
       </c>
       <c r="E92" s="4">
-        <v>0.006504629629629629</v>
+        <v>0.00986111111111111</v>
       </c>
     </row>
     <row r="93">
@@ -2512,7 +2506,7 @@
         <v>500.0</v>
       </c>
       <c r="E93" s="4">
-        <v>0.00986111111111111</v>
+        <v>0.014965277777777777</v>
       </c>
     </row>
     <row r="94">
@@ -2529,7 +2523,7 @@
         <v>500.0</v>
       </c>
       <c r="E94" s="4">
-        <v>0.014965277777777777</v>
+        <v>0.015034722222222222</v>
       </c>
     </row>
     <row r="95">
@@ -2546,7 +2540,7 @@
         <v>500.0</v>
       </c>
       <c r="E95" s="4">
-        <v>0.015034722222222222</v>
+        <v>0.016666666666666666</v>
       </c>
     </row>
     <row r="96">
@@ -2563,7 +2557,7 @@
         <v>500.0</v>
       </c>
       <c r="E96" s="4">
-        <v>0.016666666666666666</v>
+        <v>0.02140046296296296</v>
       </c>
     </row>
     <row r="97">
@@ -2580,7 +2574,7 @@
         <v>500.0</v>
       </c>
       <c r="E97" s="4">
-        <v>0.02140046296296296</v>
+        <v>0.022094907407407407</v>
       </c>
     </row>
     <row r="98">
@@ -2597,7 +2591,7 @@
         <v>500.0</v>
       </c>
       <c r="E98" s="4">
-        <v>0.022094907407407407</v>
+        <v>0.022152777777777778</v>
       </c>
     </row>
     <row r="99">
@@ -2614,15 +2608,15 @@
         <v>500.0</v>
       </c>
       <c r="E99" s="4">
-        <v>0.022152777777777778</v>
+        <v>0.025752314814814815</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B100" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="B100" s="2" t="s">
-        <v>201</v>
       </c>
       <c r="C100" s="3">
         <v>0.0</v>
@@ -2631,12 +2625,12 @@
         <v>500.0</v>
       </c>
       <c r="E100" s="4">
-        <v>0.025752314814814815</v>
+        <v>0.030428240740740742</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="s">
-        <v>37</v>
+        <v>201</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>202</v>
@@ -2648,7 +2642,7 @@
         <v>500.0</v>
       </c>
       <c r="E101" s="4">
-        <v>0.030428240740740742</v>
+        <v>0.035925925925925924</v>
       </c>
     </row>
     <row r="102">
@@ -2665,7 +2659,7 @@
         <v>500.0</v>
       </c>
       <c r="E102" s="4">
-        <v>0.035925925925925924</v>
+        <v>0.04318287037037037</v>
       </c>
     </row>
     <row r="103">
@@ -2682,7 +2676,7 @@
         <v>500.0</v>
       </c>
       <c r="E103" s="4">
-        <v>0.04318287037037037</v>
+        <v>0.046377314814814816</v>
       </c>
     </row>
     <row r="104">
@@ -2699,7 +2693,7 @@
         <v>500.0</v>
       </c>
       <c r="E104" s="4">
-        <v>0.046377314814814816</v>
+        <v>0.055219907407407405</v>
       </c>
     </row>
     <row r="105">
@@ -2716,7 +2710,7 @@
         <v>500.0</v>
       </c>
       <c r="E105" s="4">
-        <v>0.055219907407407405</v>
+        <v>0.058912037037037034</v>
       </c>
     </row>
     <row r="106">
@@ -2733,23 +2727,6 @@
         <v>500.0</v>
       </c>
       <c r="E106" s="4">
-        <v>0.058912037037037034</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="C107" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="D107" s="3">
-        <v>500.0</v>
-      </c>
-      <c r="E107" s="4">
         <v>0.06251157407407408</v>
       </c>
     </row>

</xml_diff>